<commit_message>
cuarto trimestre informacion publica
</commit_message>
<xml_diff>
--- a/assets/archivos/TRANSPARENCIA/ART 63 COMUNES 2023/4TO_TRIMESTRE/FRACC 64/LTAIPT_A64F01IG1.xlsx
+++ b/assets/archivos/TRANSPARENCIA/ART 63 COMUNES 2023/4TO_TRIMESTRE/FRACC 64/LTAIPT_A64F01IG1.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23127"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9c8ec10a61716621/Documentos/CUARTO PAG WEB/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_F5EAEF41F0BFDC4B82D1BA7230C4870788D71477" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{3B9E98A2-F077-468D-89FD-5F962A7E7116}"/>
   <bookViews>
-    <workbookView xWindow="330" yWindow="555" windowWidth="19815" windowHeight="8385"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Informacion" sheetId="1" r:id="rId1"/>
@@ -139,37 +145,37 @@
     <t>Nota</t>
   </si>
   <si>
-    <t>720DCAED160C16305C17B59024BBA95E</t>
-  </si>
-  <si>
-    <t>2022</t>
-  </si>
-  <si>
-    <t>01/07/2022</t>
-  </si>
-  <si>
-    <t>31/12/2022</t>
+    <t>2023</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>15/10/2022</t>
+    <t>15/04/2023</t>
   </si>
   <si>
     <t>Área de Transparencia</t>
   </si>
   <si>
-    <t>27/01/2023</t>
-  </si>
-  <si>
-    <t>Durante el periodo del 01 de julio de 2022 al 31 de diciembre del 2022, el Colegio de Bachilleres del Estado de Tlaxcala no cuenta por el momento con Dictámenes de Iniciativas de carácter legal, vinculadas con sus atribuciones.</t>
+    <t>11/10/2023</t>
+  </si>
+  <si>
+    <t>0C33C9733FA5EEB5888A026F1E90316E</t>
+  </si>
+  <si>
+    <t>01/10/2023</t>
+  </si>
+  <si>
+    <t>31/12/2023</t>
+  </si>
+  <si>
+    <t>Durante el periodo del 01 de octubre de 2023 al 31 de diciembre del 2023, el Colegio de Bachilleres del Estado de Tlaxcala no cuenta por el momento con Dictámenes de Iniciativas de carácter legal, de acuerdo al Artículo 64 fracción VII vinculadas con sus atribuciones.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -265,6 +271,9 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
@@ -280,44 +289,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -345,14 +354,31 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -380,6 +406,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -391,171 +434,147 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="35000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="63000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="40000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -573,7 +592,7 @@
     <col min="12" max="12" width="73.140625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="20" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="255" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="226.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
@@ -766,46 +785,46 @@
     </row>
     <row r="8" spans="1:15" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="F8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="I8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="L8" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="M8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="N8" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="M8" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>48</v>
       </c>
       <c r="O8" s="2" t="s">
         <v>49</v>

</xml_diff>